<commit_message>
Check of the folder structure
Suppression of useless file (read_me.txt)
</commit_message>
<xml_diff>
--- a/DAT/raw/data_BodyPerception_new.xlsx
+++ b/DAT/raw/data_BodyPerception_new.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/delphinehund/Desktop/Stage/Pilot_Study-SocBodPer/V2/code/DAT/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48AB290B-19CF-1949-823E-F126F4C0DC3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36477EA0-8FF6-6449-9403-5BFC0E77908A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11620" yWindow="2600" windowWidth="16380" windowHeight="16520" tabRatio="212" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -967,7 +967,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BI27"/>
+  <dimension ref="A1:BH27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -3840,7 +3840,7 @@
         <v>2.14</v>
       </c>
     </row>
-    <row r="17" spans="1:61" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:60" x14ac:dyDescent="0.15">
       <c r="A17" s="1">
         <v>959</v>
       </c>
@@ -4018,7 +4018,7 @@
         <v>1.06</v>
       </c>
     </row>
-    <row r="18" spans="1:61" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:60" x14ac:dyDescent="0.15">
       <c r="A18" s="1">
         <v>960</v>
       </c>
@@ -4196,7 +4196,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:61" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:60" x14ac:dyDescent="0.15">
       <c r="A19" s="1">
         <v>961</v>
       </c>
@@ -4374,7 +4374,7 @@
         <v>0.72</v>
       </c>
     </row>
-    <row r="20" spans="1:61" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:60" x14ac:dyDescent="0.15">
       <c r="A20" s="1">
         <v>981</v>
       </c>
@@ -4552,7 +4552,7 @@
         <v>0.64</v>
       </c>
     </row>
-    <row r="21" spans="1:61" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:60" x14ac:dyDescent="0.15">
       <c r="A21" s="1">
         <v>997</v>
       </c>
@@ -4730,7 +4730,7 @@
         <v>1.38</v>
       </c>
     </row>
-    <row r="22" spans="1:61" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:60" x14ac:dyDescent="0.15">
       <c r="A22" s="1">
         <v>998</v>
       </c>
@@ -4908,7 +4908,7 @@
         <v>1.72</v>
       </c>
     </row>
-    <row r="23" spans="1:61" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:60" x14ac:dyDescent="0.15">
       <c r="A23" s="1">
         <v>1009</v>
       </c>
@@ -5086,7 +5086,7 @@
         <v>1.23</v>
       </c>
     </row>
-    <row r="24" spans="1:61" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:60" x14ac:dyDescent="0.15">
       <c r="A24" s="1">
         <v>1030</v>
       </c>
@@ -5264,7 +5264,7 @@
         <v>0.69</v>
       </c>
     </row>
-    <row r="25" spans="1:61" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:60" x14ac:dyDescent="0.15">
       <c r="A25" s="1">
         <v>1145</v>
       </c>
@@ -5414,36 +5414,35 @@
       <c r="AY25" s="1">
         <v>242</v>
       </c>
-      <c r="AZ25" s="3"/>
-      <c r="BA25" s="3">
+      <c r="AZ25" s="3">
         <v>46104.839942129998</v>
       </c>
-      <c r="BB25" s="2" t="s">
+      <c r="BA25" s="2" t="s">
         <v>103</v>
       </c>
+      <c r="BB25" s="1">
+        <v>1</v>
+      </c>
       <c r="BC25" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BD25" s="1">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="BE25" s="1">
         <v>9</v>
       </c>
       <c r="BF25" s="1">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="BG25" s="1">
         <v>0</v>
       </c>
-      <c r="BH25" s="1">
-        <v>0</v>
-      </c>
-      <c r="BI25" s="4">
+      <c r="BH25" s="4">
         <v>2.42</v>
       </c>
     </row>
-    <row r="26" spans="1:61" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:60" x14ac:dyDescent="0.15">
       <c r="A26" s="1">
         <v>1225</v>
       </c>
@@ -5593,36 +5592,35 @@
       <c r="AY26" s="1">
         <v>305</v>
       </c>
-      <c r="AZ26" s="3"/>
-      <c r="BA26" s="3">
+      <c r="AZ26" s="3">
         <v>46105.345740741002</v>
       </c>
-      <c r="BB26" s="2" t="s">
+      <c r="BA26" s="2" t="s">
         <v>103</v>
       </c>
+      <c r="BB26" s="1">
+        <v>1</v>
+      </c>
       <c r="BC26" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BD26" s="1">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="BE26" s="1">
         <v>9</v>
       </c>
       <c r="BF26" s="1">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="BG26" s="1">
         <v>0</v>
       </c>
-      <c r="BH26" s="1">
-        <v>0</v>
-      </c>
-      <c r="BI26" s="4">
+      <c r="BH26" s="4">
         <v>2.08</v>
       </c>
     </row>
-    <row r="27" spans="1:61" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:60" x14ac:dyDescent="0.15">
       <c r="A27" s="1">
         <v>1499</v>
       </c>
@@ -5772,32 +5770,31 @@
       <c r="AY27" s="1">
         <v>299</v>
       </c>
-      <c r="AZ27" s="3"/>
-      <c r="BA27" s="3">
+      <c r="AZ27" s="3">
         <v>46118.578287037002</v>
       </c>
-      <c r="BB27" s="2" t="s">
+      <c r="BA27" s="2" t="s">
         <v>103</v>
       </c>
+      <c r="BB27" s="1">
+        <v>1</v>
+      </c>
       <c r="BC27" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BD27" s="1">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="BE27" s="1">
         <v>9</v>
       </c>
       <c r="BF27" s="1">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="BG27" s="1">
         <v>0</v>
       </c>
-      <c r="BH27" s="1">
-        <v>0</v>
-      </c>
-      <c r="BI27" s="4">
+      <c r="BH27" s="4">
         <v>0.85</v>
       </c>
     </row>

</xml_diff>